<commit_message>
Better agdis palette and fixed unset_mediocre_all()
</commit_message>
<xml_diff>
--- a/inst/data-raw/colors_table.xlsx
+++ b/inst/data-raw/colors_table.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="67">
   <si>
     <t>pal</t>
   </si>
@@ -70,27 +70,6 @@
     <t>#1B3037, #E9C46A, #28847D, #C65D44</t>
   </si>
   <si>
-    <t>green</t>
-  </si>
-  <si>
-    <t>#1B4332</t>
-  </si>
-  <si>
-    <t>#162720</t>
-  </si>
-  <si>
-    <t>#F5FAF6</t>
-  </si>
-  <si>
-    <t>#6C2B46</t>
-  </si>
-  <si>
-    <t>#D8F3DC, #C3E0C9, #AFCDB7, #9BBAA5, #87A793, #739480, #5E816E, #4A6E5C, #365C4A, #214938, #1A3F2F, #19392B, #183327, #172D23, #162720</t>
-  </si>
-  <si>
-    <t>#162720, #87A793, #D8F3DC, #214938</t>
-  </si>
-  <si>
     <t>hotcold</t>
   </si>
   <si>
@@ -223,19 +202,16 @@
     <t>agdis</t>
   </si>
   <si>
-    <t>#7A5B13</t>
-  </si>
-  <si>
-    <t>#F9EFDC</t>
-  </si>
-  <si>
-    <t>#DEBA71</t>
-  </si>
-  <si>
-    <t>#362703, #61480D, #8B6B1F, #B28F3A, #C9B482, #DBD3BF, #E6E3DC, #E7E7E7, #E2E3EA, #D0D2E4, #B0B3DE, #878CD9, #565FDE, #2D36C0, #091187</t>
-  </si>
-  <si>
-    <t>#7A5B13, #DEBA71, #050A4D, #9A9FD5</t>
+    <t>#6b5811</t>
+  </si>
+  <si>
+    <t>#fcf7ee</t>
+  </si>
+  <si>
+    <t>#EDD2A4, #E8CB95, #E4C486, #E0BD78, #D5B36A, #C5A55C, #B5974E, #A58941, #947B33, #836D25, #735F17, #62510F, #51430B, #403607, #302903</t>
+  </si>
+  <si>
+    <t>#6B5811, #EDD2A4, #110c3d, #732222</t>
   </si>
 </sst>
 </file>
@@ -1517,7 +1493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="10.8333" defaultRowHeight="16" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="13" style="1" customWidth="1"/>
@@ -1611,46 +1587,46 @@
         <v>22</v>
       </c>
       <c r="E4" t="s" s="6">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s" s="7">
         <v>23</v>
       </c>
-      <c r="F4" t="s" s="7">
+      <c r="G4" t="s" s="6">
         <v>24</v>
-      </c>
-      <c r="G4" t="s" s="6">
-        <v>25</v>
       </c>
       <c r="H4" s="8"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" t="s" s="5">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s" s="6">
         <v>26</v>
       </c>
-      <c r="B5" t="s" s="6">
+      <c r="C5" t="s" s="6">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s" s="6">
         <v>27</v>
-      </c>
-      <c r="C5" t="s" s="6">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s" s="6">
-        <v>29</v>
       </c>
       <c r="E5" t="s" s="6">
         <v>28</v>
       </c>
       <c r="F5" t="s" s="7">
+        <v>29</v>
+      </c>
+      <c r="G5" t="s" s="7">
         <v>30</v>
       </c>
-      <c r="G5" t="s" s="6">
-        <v>31</v>
-      </c>
-      <c r="H5" s="8"/>
+      <c r="H5" s="9"/>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" t="s" s="5">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s" s="6">
         <v>32</v>
-      </c>
-      <c r="B6" t="s" s="6">
-        <v>33</v>
       </c>
       <c r="C6" t="s" s="6">
         <v>33</v>
@@ -1659,33 +1635,33 @@
         <v>34</v>
       </c>
       <c r="E6" t="s" s="6">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s" s="7">
         <v>35</v>
       </c>
-      <c r="F6" t="s" s="7">
+      <c r="G6" t="s" s="7">
         <v>36</v>
       </c>
-      <c r="G6" t="s" s="7">
-        <v>37</v>
-      </c>
-      <c r="H6" s="9"/>
+      <c r="H6" s="8"/>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" t="s" s="5">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s" s="6">
         <v>38</v>
       </c>
-      <c r="B7" t="s" s="6">
+      <c r="C7" t="s" s="6">
         <v>39</v>
       </c>
-      <c r="C7" t="s" s="6">
+      <c r="D7" t="s" s="6">
         <v>40</v>
       </c>
-      <c r="D7" t="s" s="6">
+      <c r="E7" t="s" s="6">
         <v>41</v>
       </c>
-      <c r="E7" t="s" s="6">
-        <v>40</v>
-      </c>
-      <c r="F7" t="s" s="7">
+      <c r="F7" t="s" s="6">
         <v>42</v>
       </c>
       <c r="G7" t="s" s="7">
@@ -1693,7 +1669,7 @@
       </c>
       <c r="H7" s="8"/>
     </row>
-    <row r="8" ht="17" customHeight="1">
+    <row r="8" ht="15.35" customHeight="1">
       <c r="A8" t="s" s="5">
         <v>44</v>
       </c>
@@ -1704,39 +1680,39 @@
         <v>46</v>
       </c>
       <c r="D8" t="s" s="6">
+        <v>40</v>
+      </c>
+      <c r="E8" t="s" s="6">
         <v>47</v>
       </c>
-      <c r="E8" t="s" s="6">
+      <c r="F8" t="s" s="6">
         <v>48</v>
       </c>
-      <c r="F8" t="s" s="6">
+      <c r="G8" t="s" s="6">
         <v>49</v>
-      </c>
-      <c r="G8" t="s" s="7">
-        <v>50</v>
       </c>
       <c r="H8" s="8"/>
     </row>
-    <row r="9" ht="15.35" customHeight="1">
+    <row r="9" ht="17" customHeight="1">
       <c r="A9" t="s" s="5">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s" s="6">
         <v>51</v>
       </c>
-      <c r="B9" t="s" s="6">
+      <c r="C9" t="s" s="6">
         <v>52</v>
       </c>
-      <c r="C9" t="s" s="6">
+      <c r="D9" t="s" s="6">
         <v>53</v>
-      </c>
-      <c r="D9" t="s" s="6">
-        <v>47</v>
       </c>
       <c r="E9" t="s" s="6">
         <v>54</v>
       </c>
-      <c r="F9" t="s" s="6">
+      <c r="F9" t="s" s="7">
         <v>55</v>
       </c>
-      <c r="G9" t="s" s="6">
+      <c r="G9" t="s" s="7">
         <v>56</v>
       </c>
       <c r="H9" s="8"/>
@@ -1749,69 +1725,45 @@
         <v>58</v>
       </c>
       <c r="C10" t="s" s="6">
+        <v>39</v>
+      </c>
+      <c r="D10" t="s" s="6">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s" s="6">
         <v>59</v>
       </c>
-      <c r="D10" t="s" s="6">
+      <c r="F10" t="s" s="7">
         <v>60</v>
       </c>
-      <c r="E10" t="s" s="6">
+      <c r="G10" t="s" s="7">
         <v>61</v>
-      </c>
-      <c r="F10" t="s" s="7">
-        <v>62</v>
-      </c>
-      <c r="G10" t="s" s="7">
-        <v>63</v>
       </c>
       <c r="H10" s="8"/>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="A11" t="s" s="5">
+      <c r="A11" t="s" s="10">
+        <v>62</v>
+      </c>
+      <c r="B11" t="s" s="11">
+        <v>63</v>
+      </c>
+      <c r="C11" t="s" s="11">
+        <v>39</v>
+      </c>
+      <c r="D11" t="s" s="11">
         <v>64</v>
       </c>
-      <c r="B11" t="s" s="6">
+      <c r="E11" t="s" s="11">
+        <v>39</v>
+      </c>
+      <c r="F11" t="s" s="12">
         <v>65</v>
       </c>
-      <c r="C11" t="s" s="6">
-        <v>46</v>
-      </c>
-      <c r="D11" t="s" s="6">
-        <v>47</v>
-      </c>
-      <c r="E11" t="s" s="6">
+      <c r="G11" t="s" s="12">
         <v>66</v>
       </c>
-      <c r="F11" t="s" s="7">
-        <v>67</v>
-      </c>
-      <c r="G11" t="s" s="7">
-        <v>68</v>
-      </c>
-      <c r="H11" s="8"/>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" t="s" s="10">
-        <v>69</v>
-      </c>
-      <c r="B12" t="s" s="11">
-        <v>70</v>
-      </c>
-      <c r="C12" t="s" s="11">
-        <v>46</v>
-      </c>
-      <c r="D12" t="s" s="11">
-        <v>71</v>
-      </c>
-      <c r="E12" t="s" s="11">
-        <v>72</v>
-      </c>
-      <c r="F12" t="s" s="12">
-        <v>73</v>
-      </c>
-      <c r="G12" t="s" s="12">
-        <v>74</v>
-      </c>
-      <c r="H12" s="13"/>
+      <c r="H11" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>